<commit_message>
Client BOM updated for 5,100 and 1000 boards Custom supplier price added.
</commit_message>
<xml_diff>
--- a/Deliverables/BOM/LCSC BOM For Quantity 5 Boards .xlsx
+++ b/Deliverables/BOM/LCSC BOM For Quantity 5 Boards .xlsx
@@ -1,20 +1,21 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
-  <fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="14420"/>
-  <workbookPr defaultThemeVersion="153222"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="24701"/>
+  <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="G:\Github\BriacBarthes-PhoneCharger\Deliverables\BOM\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\eSpark\BriacBarthes-PhoneCharger\Deliverables\BOM\"/>
     </mc:Choice>
   </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E2CFF2A8-17F7-427E-8D5D-1559AF8C25A9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-105" yWindow="-105" windowWidth="23250" windowHeight="14010"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Briac" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="162913" concurrentCalc="0"/>
+  <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -24,7 +25,6 @@
         <xcalcf:feature name="microsoft.com:RD"/>
         <xcalcf:feature name="microsoft.com:FV"/>
         <xcalcf:feature name="microsoft.com:LET_WF"/>
-        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
       </xcalcf:calcFeatures>
     </ext>
   </extLst>
@@ -885,7 +885,7 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="3">
     <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0.0000"/>
     <numFmt numFmtId="165" formatCode="_-[$$-409]* #,##0.00_ ;_-[$$-409]* \-#,##0.00\ ;_-[$$-409]* &quot;-&quot;??_ ;_-@_ "/>
@@ -1744,19 +1744,19 @@
     <xf numFmtId="164" fontId="12" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="15" fillId="3" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="3" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="3" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -1768,14 +1768,14 @@
     <xf numFmtId="0" fontId="8" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="15" fillId="3" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="3" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="3" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -2057,7 +2057,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:U62"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
@@ -2082,27 +2082,27 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:21" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="118" t="s">
+      <c r="A1" s="126" t="s">
         <v>73</v>
       </c>
-      <c r="B1" s="119"/>
-      <c r="C1" s="119"/>
-      <c r="D1" s="119"/>
-      <c r="E1" s="119"/>
-      <c r="F1" s="119"/>
-      <c r="G1" s="119"/>
-      <c r="H1" s="119"/>
-      <c r="I1" s="119"/>
-      <c r="J1" s="119"/>
-      <c r="K1" s="119"/>
-      <c r="L1" s="119"/>
-      <c r="M1" s="119"/>
-      <c r="N1" s="119"/>
-      <c r="O1" s="119"/>
-      <c r="P1" s="119"/>
-      <c r="Q1" s="119"/>
-      <c r="R1" s="119"/>
-      <c r="S1" s="120"/>
+      <c r="B1" s="127"/>
+      <c r="C1" s="127"/>
+      <c r="D1" s="127"/>
+      <c r="E1" s="127"/>
+      <c r="F1" s="127"/>
+      <c r="G1" s="127"/>
+      <c r="H1" s="127"/>
+      <c r="I1" s="127"/>
+      <c r="J1" s="127"/>
+      <c r="K1" s="127"/>
+      <c r="L1" s="127"/>
+      <c r="M1" s="127"/>
+      <c r="N1" s="127"/>
+      <c r="O1" s="127"/>
+      <c r="P1" s="127"/>
+      <c r="Q1" s="127"/>
+      <c r="R1" s="127"/>
+      <c r="S1" s="128"/>
     </row>
     <row r="2" spans="1:21" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A2" s="2" t="s">
@@ -2167,7 +2167,7 @@
       <c r="A3" s="12">
         <v>1</v>
       </c>
-      <c r="B3" s="122" t="s">
+      <c r="B3" s="121" t="s">
         <v>14</v>
       </c>
       <c r="C3" s="19" t="s">
@@ -2229,7 +2229,7 @@
       <c r="A4" s="12">
         <v>2</v>
       </c>
-      <c r="B4" s="121"/>
+      <c r="B4" s="122"/>
       <c r="C4" s="23" t="s">
         <v>81</v>
       </c>
@@ -2289,7 +2289,7 @@
       <c r="A5" s="12">
         <v>3</v>
       </c>
-      <c r="B5" s="121"/>
+      <c r="B5" s="122"/>
       <c r="C5" s="23" t="s">
         <v>85</v>
       </c>
@@ -2341,7 +2341,7 @@
         <f t="shared" si="2"/>
         <v>9.6</v>
       </c>
-      <c r="S5" s="126"/>
+      <c r="S5" s="118"/>
       <c r="T5" s="3"/>
       <c r="U5" s="3"/>
     </row>
@@ -2349,7 +2349,7 @@
       <c r="A6" s="12">
         <v>4</v>
       </c>
-      <c r="B6" s="121"/>
+      <c r="B6" s="122"/>
       <c r="C6" s="23" t="s">
         <v>88</v>
       </c>
@@ -2409,7 +2409,7 @@
       <c r="A7" s="12">
         <v>5</v>
       </c>
-      <c r="B7" s="121"/>
+      <c r="B7" s="122"/>
       <c r="C7" s="23" t="s">
         <v>90</v>
       </c>
@@ -2469,7 +2469,7 @@
       <c r="A8" s="12">
         <v>6</v>
       </c>
-      <c r="B8" s="121"/>
+      <c r="B8" s="122"/>
       <c r="C8" s="23" t="s">
         <v>93</v>
       </c>
@@ -2529,7 +2529,7 @@
       <c r="A9" s="12">
         <v>7</v>
       </c>
-      <c r="B9" s="121"/>
+      <c r="B9" s="122"/>
       <c r="C9" s="23" t="s">
         <v>97</v>
       </c>
@@ -2649,7 +2649,7 @@
       <c r="A11" s="12">
         <v>9</v>
       </c>
-      <c r="B11" s="121" t="s">
+      <c r="B11" s="122" t="s">
         <v>15</v>
       </c>
       <c r="C11" s="109" t="s">
@@ -2711,7 +2711,7 @@
       <c r="A12" s="12">
         <v>10</v>
       </c>
-      <c r="B12" s="121"/>
+      <c r="B12" s="122"/>
       <c r="C12" s="23" t="s">
         <v>105</v>
       </c>
@@ -2771,7 +2771,7 @@
       <c r="A13" s="12">
         <v>11</v>
       </c>
-      <c r="B13" s="121"/>
+      <c r="B13" s="122"/>
       <c r="C13" s="46" t="s">
         <v>108</v>
       </c>
@@ -2831,7 +2831,7 @@
       <c r="A14" s="12">
         <v>12</v>
       </c>
-      <c r="B14" s="122" t="s">
+      <c r="B14" s="121" t="s">
         <v>29</v>
       </c>
       <c r="C14" s="53" t="s">
@@ -2893,7 +2893,7 @@
       <c r="A15" s="12">
         <v>13</v>
       </c>
-      <c r="B15" s="121"/>
+      <c r="B15" s="122"/>
       <c r="C15" s="60" t="s">
         <v>213</v>
       </c>
@@ -2945,7 +2945,7 @@
         <f t="shared" si="2"/>
         <v>6.4</v>
       </c>
-      <c r="S15" s="126"/>
+      <c r="S15" s="118"/>
       <c r="T15" s="17"/>
       <c r="U15" s="17"/>
     </row>
@@ -3013,7 +3013,7 @@
       <c r="A17" s="12">
         <v>15</v>
       </c>
-      <c r="B17" s="121" t="s">
+      <c r="B17" s="122" t="s">
         <v>69</v>
       </c>
       <c r="C17" s="63" t="s">
@@ -3075,7 +3075,7 @@
       <c r="A18" s="12">
         <v>16</v>
       </c>
-      <c r="B18" s="121"/>
+      <c r="B18" s="122"/>
       <c r="C18" s="46" t="s">
         <v>119</v>
       </c>
@@ -3125,7 +3125,7 @@
       <c r="A19" s="12">
         <v>17</v>
       </c>
-      <c r="B19" s="122" t="s">
+      <c r="B19" s="121" t="s">
         <v>26</v>
       </c>
       <c r="C19" s="53" t="s">
@@ -3187,7 +3187,7 @@
       <c r="A20" s="12">
         <v>18</v>
       </c>
-      <c r="B20" s="121"/>
+      <c r="B20" s="122"/>
       <c r="C20" s="23" t="s">
         <v>124</v>
       </c>
@@ -3299,7 +3299,7 @@
         <f t="shared" si="2"/>
         <v>5.0960000000000001</v>
       </c>
-      <c r="S21" s="127"/>
+      <c r="S21" s="119"/>
       <c r="T21" s="3"/>
       <c r="U21" s="3"/>
     </row>
@@ -3307,7 +3307,7 @@
       <c r="A22" s="12">
         <v>20</v>
       </c>
-      <c r="B22" s="122" t="s">
+      <c r="B22" s="121" t="s">
         <v>16</v>
       </c>
       <c r="C22" s="53" t="s">
@@ -3369,7 +3369,7 @@
       <c r="A23" s="12">
         <v>21</v>
       </c>
-      <c r="B23" s="121"/>
+      <c r="B23" s="122"/>
       <c r="C23" s="23" t="s">
         <v>132</v>
       </c>
@@ -3429,7 +3429,7 @@
       <c r="A24" s="12">
         <v>22</v>
       </c>
-      <c r="B24" s="121"/>
+      <c r="B24" s="122"/>
       <c r="C24" s="23" t="s">
         <v>135</v>
       </c>
@@ -3489,7 +3489,7 @@
       <c r="A25" s="12">
         <v>23</v>
       </c>
-      <c r="B25" s="121"/>
+      <c r="B25" s="122"/>
       <c r="C25" s="23" t="s">
         <v>137</v>
       </c>
@@ -3549,7 +3549,7 @@
       <c r="A26" s="12">
         <v>24</v>
       </c>
-      <c r="B26" s="121"/>
+      <c r="B26" s="122"/>
       <c r="C26" s="23" t="s">
         <v>139</v>
       </c>
@@ -3609,7 +3609,7 @@
       <c r="A27" s="12">
         <v>25</v>
       </c>
-      <c r="B27" s="121"/>
+      <c r="B27" s="122"/>
       <c r="C27" s="23" t="s">
         <v>142</v>
       </c>
@@ -3669,7 +3669,7 @@
       <c r="A28" s="12">
         <v>26</v>
       </c>
-      <c r="B28" s="121"/>
+      <c r="B28" s="122"/>
       <c r="C28" s="23" t="s">
         <v>146</v>
       </c>
@@ -3729,7 +3729,7 @@
       <c r="A29" s="12">
         <v>27</v>
       </c>
-      <c r="B29" s="121"/>
+      <c r="B29" s="122"/>
       <c r="C29" s="60" t="s">
         <v>220</v>
       </c>
@@ -3789,7 +3789,7 @@
       <c r="A30" s="12">
         <v>28</v>
       </c>
-      <c r="B30" s="121"/>
+      <c r="B30" s="122"/>
       <c r="C30" s="23" t="s">
         <v>149</v>
       </c>
@@ -3849,7 +3849,7 @@
       <c r="A31" s="12">
         <v>29</v>
       </c>
-      <c r="B31" s="121"/>
+      <c r="B31" s="122"/>
       <c r="C31" s="23" t="s">
         <v>152</v>
       </c>
@@ -3909,7 +3909,7 @@
       <c r="A32" s="12">
         <v>30</v>
       </c>
-      <c r="B32" s="121"/>
+      <c r="B32" s="122"/>
       <c r="C32" s="60" t="s">
         <v>262</v>
       </c>
@@ -3969,7 +3969,7 @@
       <c r="A33" s="12">
         <v>31</v>
       </c>
-      <c r="B33" s="121"/>
+      <c r="B33" s="122"/>
       <c r="C33" s="60" t="s">
         <v>221</v>
       </c>
@@ -4029,7 +4029,7 @@
       <c r="A34" s="12">
         <v>32</v>
       </c>
-      <c r="B34" s="121"/>
+      <c r="B34" s="122"/>
       <c r="C34" s="23" t="s">
         <v>156</v>
       </c>
@@ -4149,7 +4149,7 @@
       <c r="A36" s="12">
         <v>34</v>
       </c>
-      <c r="B36" s="121" t="s">
+      <c r="B36" s="122" t="s">
         <v>70</v>
       </c>
       <c r="C36" s="63" t="s">
@@ -4211,7 +4211,7 @@
       <c r="A37" s="12">
         <v>35</v>
       </c>
-      <c r="B37" s="121"/>
+      <c r="B37" s="122"/>
       <c r="C37" s="73" t="s">
         <v>222</v>
       </c>
@@ -4271,7 +4271,7 @@
       <c r="A38" s="12">
         <v>36</v>
       </c>
-      <c r="B38" s="122" t="s">
+      <c r="B38" s="121" t="s">
         <v>71</v>
       </c>
       <c r="C38" s="53" t="s">
@@ -4333,7 +4333,7 @@
       <c r="A39" s="12">
         <v>37</v>
       </c>
-      <c r="B39" s="121"/>
+      <c r="B39" s="122"/>
       <c r="C39" s="23" t="s">
         <v>176</v>
       </c>
@@ -4393,7 +4393,7 @@
       <c r="A40" s="12">
         <v>38</v>
       </c>
-      <c r="B40" s="121"/>
+      <c r="B40" s="122"/>
       <c r="C40" s="60" t="s">
         <v>271</v>
       </c>
@@ -4445,7 +4445,7 @@
         <f t="shared" si="2"/>
         <v>6.6899999999999995</v>
       </c>
-      <c r="S40" s="126"/>
+      <c r="S40" s="118"/>
       <c r="T40" s="3"/>
       <c r="U40" s="3"/>
     </row>
@@ -4453,7 +4453,7 @@
       <c r="A41" s="12">
         <v>39</v>
       </c>
-      <c r="B41" s="121"/>
+      <c r="B41" s="122"/>
       <c r="C41" s="23" t="s">
         <v>179</v>
       </c>
@@ -4505,7 +4505,7 @@
         <f t="shared" si="2"/>
         <v>12.426000000000002</v>
       </c>
-      <c r="S41" s="126"/>
+      <c r="S41" s="118"/>
       <c r="T41" s="3"/>
       <c r="U41" s="3"/>
     </row>
@@ -4513,7 +4513,7 @@
       <c r="A42" s="12">
         <v>40</v>
       </c>
-      <c r="B42" s="121"/>
+      <c r="B42" s="122"/>
       <c r="C42" s="60" t="s">
         <v>229</v>
       </c>
@@ -4565,7 +4565,7 @@
         <f t="shared" si="2"/>
         <v>2.8679999999999999</v>
       </c>
-      <c r="S42" s="126"/>
+      <c r="S42" s="118"/>
       <c r="T42" s="3"/>
       <c r="U42" s="3"/>
     </row>
@@ -4573,7 +4573,7 @@
       <c r="A43" s="12">
         <v>41</v>
       </c>
-      <c r="B43" s="121"/>
+      <c r="B43" s="122"/>
       <c r="C43" s="60" t="s">
         <v>67</v>
       </c>
@@ -4625,7 +4625,7 @@
         <f t="shared" si="2"/>
         <v>3.8220000000000001</v>
       </c>
-      <c r="S43" s="126"/>
+      <c r="S43" s="118"/>
       <c r="T43" s="3"/>
       <c r="U43" s="3"/>
     </row>
@@ -4633,7 +4633,7 @@
       <c r="A44" s="12">
         <v>42</v>
       </c>
-      <c r="B44" s="121"/>
+      <c r="B44" s="122"/>
       <c r="C44" s="60" t="s">
         <v>232</v>
       </c>
@@ -4685,7 +4685,7 @@
         <f t="shared" si="2"/>
         <v>19.11</v>
       </c>
-      <c r="S44" s="126"/>
+      <c r="S44" s="118"/>
       <c r="T44" s="3"/>
       <c r="U44" s="3"/>
     </row>
@@ -4693,7 +4693,7 @@
       <c r="A45" s="12">
         <v>43</v>
       </c>
-      <c r="B45" s="121"/>
+      <c r="B45" s="122"/>
       <c r="C45" s="60" t="s">
         <v>236</v>
       </c>
@@ -4745,7 +4745,7 @@
         <f t="shared" si="2"/>
         <v>19.11</v>
       </c>
-      <c r="S45" s="126"/>
+      <c r="S45" s="118"/>
       <c r="T45" s="3"/>
       <c r="U45" s="3"/>
     </row>
@@ -4805,7 +4805,7 @@
         <f t="shared" si="2"/>
         <v>5.7359999999999998</v>
       </c>
-      <c r="S46" s="127"/>
+      <c r="S46" s="119"/>
       <c r="T46" s="3"/>
       <c r="U46" s="3"/>
     </row>
@@ -4875,7 +4875,7 @@
       <c r="A48" s="12">
         <v>46</v>
       </c>
-      <c r="B48" s="122" t="s">
+      <c r="B48" s="121" t="s">
         <v>72</v>
       </c>
       <c r="C48" s="53" t="s">
@@ -4919,7 +4919,7 @@
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
-      <c r="S48" s="128"/>
+      <c r="S48" s="120"/>
       <c r="T48" s="3"/>
       <c r="U48" s="3"/>
     </row>
@@ -4927,7 +4927,7 @@
       <c r="A49" s="12">
         <v>47</v>
       </c>
-      <c r="B49" s="121"/>
+      <c r="B49" s="122"/>
       <c r="C49" s="23" t="s">
         <v>191</v>
       </c>
@@ -4987,7 +4987,7 @@
       <c r="A50" s="12">
         <v>48</v>
       </c>
-      <c r="B50" s="121"/>
+      <c r="B50" s="122"/>
       <c r="C50" s="23" t="s">
         <v>194</v>
       </c>
@@ -5047,7 +5047,7 @@
       <c r="A51" s="12">
         <v>49</v>
       </c>
-      <c r="B51" s="121"/>
+      <c r="B51" s="122"/>
       <c r="C51" s="23" t="s">
         <v>197</v>
       </c>
@@ -5228,6 +5228,11 @@
     </row>
   </sheetData>
   <mergeCells count="12">
+    <mergeCell ref="A1:S1"/>
+    <mergeCell ref="B11:B13"/>
+    <mergeCell ref="B3:B10"/>
+    <mergeCell ref="B14:B16"/>
+    <mergeCell ref="B17:B18"/>
     <mergeCell ref="B48:B52"/>
     <mergeCell ref="M53:N53"/>
     <mergeCell ref="M54:N54"/>
@@ -5235,11 +5240,6 @@
     <mergeCell ref="B36:B37"/>
     <mergeCell ref="B38:B46"/>
     <mergeCell ref="B22:B35"/>
-    <mergeCell ref="A1:S1"/>
-    <mergeCell ref="B11:B13"/>
-    <mergeCell ref="B3:B10"/>
-    <mergeCell ref="B14:B16"/>
-    <mergeCell ref="B17:B18"/>
   </mergeCells>
   <conditionalFormatting sqref="S19:S20">
     <cfRule type="dataBar" priority="23">
@@ -5322,44 +5322,44 @@
     </cfRule>
   </conditionalFormatting>
   <hyperlinks>
-    <hyperlink ref="N11" r:id="rId1"/>
-    <hyperlink ref="N12" r:id="rId2"/>
-    <hyperlink ref="N14" r:id="rId3"/>
-    <hyperlink ref="N17" r:id="rId4"/>
-    <hyperlink ref="N20" r:id="rId5"/>
-    <hyperlink ref="N25" r:id="rId6"/>
-    <hyperlink ref="N27" r:id="rId7"/>
-    <hyperlink ref="N36" r:id="rId8"/>
-    <hyperlink ref="N39" r:id="rId9"/>
-    <hyperlink ref="N47" r:id="rId10"/>
-    <hyperlink ref="N49" r:id="rId11"/>
-    <hyperlink ref="N50" r:id="rId12"/>
-    <hyperlink ref="N9" r:id="rId13"/>
-    <hyperlink ref="N3" r:id="rId14"/>
-    <hyperlink ref="N6" r:id="rId15"/>
-    <hyperlink ref="N7" r:id="rId16"/>
-    <hyperlink ref="N13" r:id="rId17"/>
-    <hyperlink ref="N16" r:id="rId18"/>
-    <hyperlink ref="N22" r:id="rId19"/>
-    <hyperlink ref="N23" r:id="rId20"/>
-    <hyperlink ref="N26" r:id="rId21"/>
-    <hyperlink ref="N28" r:id="rId22"/>
-    <hyperlink ref="N29" r:id="rId23"/>
-    <hyperlink ref="N30" r:id="rId24"/>
-    <hyperlink ref="N31" r:id="rId25"/>
-    <hyperlink ref="N33" r:id="rId26"/>
-    <hyperlink ref="N34" r:id="rId27"/>
-    <hyperlink ref="N35" r:id="rId28"/>
-    <hyperlink ref="N24" r:id="rId29"/>
-    <hyperlink ref="N8" r:id="rId30"/>
-    <hyperlink ref="N10" r:id="rId31"/>
-    <hyperlink ref="N32" r:id="rId32"/>
-    <hyperlink ref="N51" r:id="rId33"/>
-    <hyperlink ref="N4" r:id="rId34"/>
-    <hyperlink ref="N19" r:id="rId35"/>
-    <hyperlink ref="N38" r:id="rId36"/>
-    <hyperlink ref="N52" r:id="rId37"/>
-    <hyperlink ref="N37" r:id="rId38"/>
+    <hyperlink ref="N11" r:id="rId1" xr:uid="{00000000-0004-0000-0000-000000000000}"/>
+    <hyperlink ref="N12" r:id="rId2" xr:uid="{00000000-0004-0000-0000-000001000000}"/>
+    <hyperlink ref="N14" r:id="rId3" xr:uid="{00000000-0004-0000-0000-000002000000}"/>
+    <hyperlink ref="N17" r:id="rId4" xr:uid="{00000000-0004-0000-0000-000003000000}"/>
+    <hyperlink ref="N20" r:id="rId5" xr:uid="{00000000-0004-0000-0000-000004000000}"/>
+    <hyperlink ref="N25" r:id="rId6" xr:uid="{00000000-0004-0000-0000-000005000000}"/>
+    <hyperlink ref="N27" r:id="rId7" xr:uid="{00000000-0004-0000-0000-000006000000}"/>
+    <hyperlink ref="N36" r:id="rId8" xr:uid="{00000000-0004-0000-0000-000007000000}"/>
+    <hyperlink ref="N39" r:id="rId9" xr:uid="{00000000-0004-0000-0000-000008000000}"/>
+    <hyperlink ref="N47" r:id="rId10" xr:uid="{00000000-0004-0000-0000-000009000000}"/>
+    <hyperlink ref="N49" r:id="rId11" xr:uid="{00000000-0004-0000-0000-00000A000000}"/>
+    <hyperlink ref="N50" r:id="rId12" xr:uid="{00000000-0004-0000-0000-00000B000000}"/>
+    <hyperlink ref="N9" r:id="rId13" xr:uid="{00000000-0004-0000-0000-00000C000000}"/>
+    <hyperlink ref="N3" r:id="rId14" xr:uid="{00000000-0004-0000-0000-00000D000000}"/>
+    <hyperlink ref="N6" r:id="rId15" xr:uid="{00000000-0004-0000-0000-00000E000000}"/>
+    <hyperlink ref="N7" r:id="rId16" xr:uid="{00000000-0004-0000-0000-00000F000000}"/>
+    <hyperlink ref="N13" r:id="rId17" xr:uid="{00000000-0004-0000-0000-000010000000}"/>
+    <hyperlink ref="N16" r:id="rId18" xr:uid="{00000000-0004-0000-0000-000011000000}"/>
+    <hyperlink ref="N22" r:id="rId19" xr:uid="{00000000-0004-0000-0000-000012000000}"/>
+    <hyperlink ref="N23" r:id="rId20" xr:uid="{00000000-0004-0000-0000-000013000000}"/>
+    <hyperlink ref="N26" r:id="rId21" xr:uid="{00000000-0004-0000-0000-000014000000}"/>
+    <hyperlink ref="N28" r:id="rId22" xr:uid="{00000000-0004-0000-0000-000015000000}"/>
+    <hyperlink ref="N29" r:id="rId23" xr:uid="{00000000-0004-0000-0000-000016000000}"/>
+    <hyperlink ref="N30" r:id="rId24" xr:uid="{00000000-0004-0000-0000-000017000000}"/>
+    <hyperlink ref="N31" r:id="rId25" xr:uid="{00000000-0004-0000-0000-000018000000}"/>
+    <hyperlink ref="N33" r:id="rId26" xr:uid="{00000000-0004-0000-0000-000019000000}"/>
+    <hyperlink ref="N34" r:id="rId27" xr:uid="{00000000-0004-0000-0000-00001A000000}"/>
+    <hyperlink ref="N35" r:id="rId28" xr:uid="{00000000-0004-0000-0000-00001B000000}"/>
+    <hyperlink ref="N24" r:id="rId29" xr:uid="{00000000-0004-0000-0000-00001C000000}"/>
+    <hyperlink ref="N8" r:id="rId30" xr:uid="{00000000-0004-0000-0000-00001D000000}"/>
+    <hyperlink ref="N10" r:id="rId31" xr:uid="{00000000-0004-0000-0000-00001E000000}"/>
+    <hyperlink ref="N32" r:id="rId32" xr:uid="{00000000-0004-0000-0000-00001F000000}"/>
+    <hyperlink ref="N51" r:id="rId33" xr:uid="{00000000-0004-0000-0000-000020000000}"/>
+    <hyperlink ref="N4" r:id="rId34" xr:uid="{00000000-0004-0000-0000-000021000000}"/>
+    <hyperlink ref="N19" r:id="rId35" xr:uid="{00000000-0004-0000-0000-000022000000}"/>
+    <hyperlink ref="N38" r:id="rId36" xr:uid="{00000000-0004-0000-0000-000023000000}"/>
+    <hyperlink ref="N52" r:id="rId37" xr:uid="{00000000-0004-0000-0000-000024000000}"/>
+    <hyperlink ref="N37" r:id="rId38" xr:uid="{00000000-0004-0000-0000-000025000000}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId39"/>

</xml_diff>